<commit_message>
auto: add 02-Knowledge (3), delete 02-Knowledge (1), modify (root) (1), modify 02-Knowledge (3)
</commit_message>
<xml_diff>
--- a/02-Knowledge/investment-research/credit-card-management/信用卡主控表.xlsx
+++ b/02-Knowledge/investment-research/credit-card-management/信用卡主控表.xlsx
@@ -219,7 +219,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -322,11 +322,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -435,6 +463,11 @@
     <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -3571,35 +3604,21 @@
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="25">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="44" t="inlineStr">
         <is>
           <t>宁波</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>贵宾厅</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="B16" s="28" t="n"/>
+      <c r="C16" s="28" t="n"/>
+      <c r="D16" s="28" t="n"/>
+      <c r="E16" s="29" t="n"/>
+      <c r="F16" s="44" t="inlineStr">
         <is>
           <t>50-80</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>600-960</t>
-        </is>
-      </c>
+      <c r="G16" s="29" t="n"/>
       <c r="H16" s="8" t="inlineStr">
         <is>
           <t>实名</t>
@@ -3612,16 +3631,25 @@
           <t>合计</t>
         </is>
       </c>
-      <c r="B17" s="39" t="n"/>
-      <c r="C17" s="39" t="n"/>
-      <c r="D17" s="39" t="n"/>
-      <c r="E17" s="39" t="n"/>
+      <c r="B17" s="45" t="n"/>
+      <c r="C17">
+        <f>SUM(C5:C15)</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>SUM(D5:D15)</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>SUM(E5:E15)</f>
+        <v/>
+      </c>
       <c r="F17" s="38" t="inlineStr">
         <is>
           <t>3,150-5,468 元</t>
         </is>
       </c>
-      <c r="G17" s="39" t="n"/>
+      <c r="G17" s="45" t="n"/>
       <c r="H17" s="40" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="25"/>
@@ -3776,8 +3804,8 @@
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="F16:G16"/>
+    <mergeCell ref="A17:B17"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A17:E17"/>
     <mergeCell ref="F17:G17"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:E15">
@@ -4267,11 +4295,7 @@
           <t>光大</t>
         </is>
       </c>
-      <c r="B8" s="37" t="inlineStr">
-        <is>
-          <t>阳光车主</t>
-        </is>
-      </c>
+      <c r="B8" s="45" t="n"/>
       <c r="C8" s="37" t="n">
         <v>500</v>
       </c>
@@ -4323,6 +4347,11 @@
     </row>
     <row r="10" ht="15" customHeight="1" s="25">
       <c r="A10" s="41" t="inlineStr"/>
+      <c r="B10" s="46" t="n"/>
+      <c r="C10" s="46" t="n"/>
+      <c r="D10" s="46" t="n"/>
+      <c r="E10" s="46" t="n"/>
+      <c r="F10" s="45" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="38" t="inlineStr">
@@ -4330,7 +4359,7 @@
           <t>合计</t>
         </is>
       </c>
-      <c r="B11" s="39" t="n"/>
+      <c r="B11" s="45" t="n"/>
       <c r="C11" s="38">
         <f>SUM(C5:C9)</f>
         <v/>
@@ -4413,19 +4442,16 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="44" t="inlineStr">
         <is>
           <t>活动返现</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="B17" s="28" t="n"/>
+      <c r="C17" s="28" t="n"/>
+      <c r="D17" s="28" t="n"/>
+      <c r="E17" s="28" t="n"/>
+      <c r="F17" s="29" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="11" t="inlineStr">
@@ -4498,16 +4524,16 @@
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="25">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="44" t="inlineStr">
         <is>
           <t>预估收入</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>2,850-4,988 元</t>
-        </is>
-      </c>
+      <c r="B23" s="28" t="n"/>
+      <c r="C23" s="28" t="n"/>
+      <c r="D23" s="28" t="n"/>
+      <c r="E23" s="28" t="n"/>
+      <c r="F23" s="29" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -4521,7 +4547,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
@@ -4533,8 +4558,8 @@
   <mergeCells count="7">
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A8:B8"/>

</xml_diff>